<commit_message>
feat(F-NAR-019): ATOM-COL.POL.001-12 Le panier de Mila
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-12.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-12.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>L'œuf encore chaud de Mila</t>
+          <t>Le panier de Mila</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cour de ferme, paille, puis cuisine</t>
+          <t>marché, chat sous table, caisse de fromages, petite balance, panier</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut un œuf encore chaud pour le gâteau. À la poule, puis au lait de chèvre, elle dit bonjour, s'il te plaît, merci.</t>
+          <t>Une moustache du chat touche le pied de table. Sur le bord, un éclat de panier brille. Mila veut le rond pâle maintenant. Elle parle trop vite, sans le mot : la dame n'a pas levé les yeux. Elle refuse de foncer, dit bonjour. Merci vécu. Le panier penche vers le chat. Un éclat de panier reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La paille pique un peu sous les sandales. Une poule rousse picore près du seau. Le seau sent le grain, tout sec. Le soleil chauffe le bois de la porte. Une plume reste collée au loquet. Tu as vu la plume, Mila ? Elle est douce. Elle est un peu chaude. Le soleil l'a chauffée. Je veux un œuf. Pour le gâteau de papa. Un œuf encore chaud, alors. La cour sent le foin coupé. Une goutte tombe du robinet de zinc. Elle fait un rond dans la poussière. On marche doucement. La poule est près du nid. En ce moment, Mila tient le petit panier. Le panier sent encore le linge propre. Un torchon blanc est plié au fond. La dame de la ferme essuie ses mains. Elle a de la paille sur le tablier. On attend un peu. Elle range le grain. Le nid est là. Il est dans l'ombre. Oui. Un œuf brun brille sous la paille. Il a des taches plus claires. Celui-là. Il est tout rond. La dame pose le seau. Elle se tourne vers elles. Tu demandes, Mila. L'œuf attend dans la paille.</t>
+          <t>Une moustache du chat touche le pied de table. Le chat dort, rond, sous le bois. Sa queue frôle une caisse de fromages. Ça sent le lait, et un peu le foin. Ça sent le lait, papa. Tu le sens, toi ? Oui, et le foin. Le soleil touche tes joues. Elles sont tièdes, maman. Papa tient la main de Mila. Sa paume sent un peu le foin. Tu as du foin, Mila ? Un peu, papa. Maman tend le panier, vide et léger. Il est léger, maman. Parce qu'il est vide. Tu as vu le chat, Mila ? Il dort sous la table. On le laisse. Des voix passent, plus loin, sur la place. Une petite balance fait tic, près de la caisse. Elle fait tic, maman. C'est la balance, près des ronds. Le bois de la table sent le soleil. Il est chaud, maman. Et le plateau, lui, est froid. Un filet de soleil tombe sur le bord. Sur le bord, un éclat de panier brille. Il brille, papa ! Tu le vois, sur le panier ? Oui, près du bord. Les ronds de la caisse sont pâles, un peu froids. Celui-là, papa. Celui près de la queue ? Oui, le pâle. Je le veux, maintenant. En ce moment, Mila avance vers la table. La dame essuie le plateau de la balance. Le métal est froid, malgré le soleil. Celui-là ! Mila parle trop vite vers la table. Sa voix se mélange au tic de la balance. La dame n'a pas levé les yeux. Oh. Le rond pâle reste dans la caisse. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le prends ! Le fromage est sur la table. Tu le vois, Mila ? Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La paille pique un peu sous les sandales. Une poule rousse picore près du seau. Le seau sent le grain, tout sec. Le soleil chauffe le bois de la porte. Une plume reste collée au loquet. Tu as vu la plume, Mila ? Elle est douce. Elle est un peu chaude. Le soleil l'a chauffée. Je veux un œuf. Pour le gâteau de papa. Un œuf encore chaud, alors. La cour sent le foin coupé. Une goutte tombe du robinet de zinc. Elle fait un rond dans la poussière. On marche doucement. La poule est près du nid. En ce moment, Mila tient le petit panier. Le panier sent encore le linge propre. Un torchon blanc est plié au fond. La dame de la ferme essuie ses mains. Elle a de la paille sur le tablier. On attend un peu. Elle range le grain. Le nid est là. Il est dans l'ombre. Oui. Un œuf brun brille sous la paille. Il a des taches plus claires. Celui-là. Il est tout rond. La dame pose le seau. Elle se tourne vers elles. Tu demandes, Mila. L'œuf attend dans la paille.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une moustache du chat touche le pied de table. Le chat dort, rond, sous le bois. Sa queue frôle une caisse de fromages. Ça sent le lait, et un peu le foin. Ça sent le lait, papa. Tu le sens, toi ? Oui, et le foin. Le soleil touche tes joues. Elles sont tièdes, maman. Papa tient la main de Mila. Sa paume sent un peu le foin. Tu as du foin, Mila ? Un peu, papa. Maman tend le panier, vide et léger. Il est léger, maman. Parce qu'il est vide. Tu as vu le chat, Mila ? Il dort sous la table. On le laisse. Des voix passent, plus loin, sur la place. Une petite balance fait tic, près de la caisse. Elle fait tic, maman. C'est la balance, près des ronds. Le bois de la table sent le soleil. Il est chaud, maman. Et le plateau, lui, est froid. Un filet de soleil tombe sur le bord. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de panier&lt;/emphasis&gt; brille. Il brille, papa ! Tu le vois, sur le panier ? Oui, près du bord. Les ronds de la caisse sont pâles, un peu froids. Celui-là, papa. Celui près de la queue ? Oui, le pâle. Je le veux, maintenant. En ce moment, Mila avance vers la table. La dame essuie le plateau de la balance. Le métal est froid, malgré le soleil. Celui-là ! Mila parle trop vite vers la table. Sa voix se mélange au tic de la balance. La dame n'a pas levé les yeux. Oh. Le rond pâle reste dans la caisse. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le prends ! Le fromage est sur la table. Tu le vois, Mila ? Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Honoré arrive au marché avec maman. Il sent les fromages. Honoré dit : &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. La dame sourit. Honoré dit : un morceau, s'il te plaît. La dame tend le sachet. Honoré dit : merci. Maman dit : bonjour, s'il te plaît, merci. Plus tard, ils passent au stand des pommes. Honoré se souvient. Il dit : bonjour. Puis : une pomme, s'il te plaît. Puis : merci. Maman dit : tu as repris les trois mots. Bonjour. S'il te plaît. Merci. Même leçon, autre stand. Honoré tient le sachet. La pomme sent le sucré. [pause]</t>
+          <t>Une moustache du chat touche le pied de table. Le chat dort, rond, sous le bois. Sa queue frôle une caisse de fromages. Ça sent le lait, et un peu le foin. Ça sent le lait, papa. Tu le sens, toi ? Oui, et le foin. Le soleil touche tes joues. Elles sont tièdes, maman. Papa tient la main de Mila. Sa paume sent un peu le foin. Tu as du foin, Mila ? Un peu, papa. Maman tend le panier, vide et léger. Il est léger, maman. Parce qu'il est vide. Tu as vu le chat, Mila ? Il dort sous la table. On le laisse. Des voix passent, plus loin, sur la place. Une petite balance fait tic, près de la caisse. Elle fait tic, maman. C'est la balance, près des ronds. Le bois de la table sent le soleil. Il est chaud, maman. Et le plateau, lui, est froid. Un filet de soleil tombe sur le bord. Sur le bord, un &lt;emphasis&gt;éclat de panier&lt;/emphasis&gt; brille. Il brille, papa ! Tu le vois, sur le panier ? Oui, près du bord. Les ronds de la caisse sont pâles, un peu froids. Celui-là, papa. Celui près de la queue ? Oui, le pâle. Je le veux, maintenant. En ce moment, Mila avance vers la table. La dame essuie le plateau de la balance. Le métal est froid, malgré le soleil. Celui-là ! Mila parle trop vite vers la table. Sa voix se mélange au tic de la balance. La dame n'a pas levé les yeux. Oh. Le rond pâle reste dans la caisse. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le prends ! Le fromage est sur la table. Tu le vois, Mila ? Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>éclat de panier</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,49 +1326,71 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_rond_pale_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La paille pique un peu sous les sandales.
-narrateur|Une poule rousse picore près du seau.
-narrateur|Le seau sent le grain, tout sec.
-narrateur|Le soleil chauffe le bois de la porte.
-narrateur|Une plume reste collée au loquet.
-maman|Tu as vu la plume, Mila ?
-enfant-f|Elle est douce.
-enfant-f|Elle est un peu chaude.
-maman|Le soleil l'a chauffée.
-enfant-f|Je veux un œuf.
-enfant-f|Pour le gâteau de papa.
-maman|Un œuf encore chaud, alors.
-narrateur|La cour sent le foin coupé.
-narrateur|Une goutte tombe du robinet de zinc.
-narrateur|Elle fait un rond dans la poussière.
-maman|On marche doucement.
-maman|La poule est près du nid.
-narrateur|En ce moment, Mila tient le petit panier.
-narrateur|Le panier sent encore le linge propre.
-narrateur|Un torchon blanc est plié au fond.
-narrateur|La dame de la ferme essuie ses mains.
-narrateur|Elle a de la paille sur le tablier.
-maman|On attend un peu.
-maman|Elle range le grain.
-enfant-f|Le nid est là.
-enfant-f|Il est dans l'ombre.
-maman|Oui.
-narrateur|Un œuf brun brille sous la paille.
-narrateur|Il a des taches plus claires.
-enfant-f|Celui-là.
-enfant-f|Il est tout rond.
-narrateur|La dame pose le seau.
-narrateur|Elle se tourne vers elles.
-maman|Tu demandes, Mila.
-narrateur|L'œuf attend dans la paille.</t>
+          <t>narrateur|Une moustache du chat touche le pied de table.
+narrateur|Le chat dort, rond, sous le bois.
+narrateur|Sa queue frôle une caisse de fromages.
+narrateur|Ça sent le lait, et un peu le foin.
+enfant-f|Ça sent le lait, papa.
+papa|Tu le sens, toi ?
+enfant-f|Oui, et le foin.
+maman|Le soleil touche tes joues.
+enfant-f|Elles sont tièdes, maman.
+narrateur|Papa tient la main de Mila.
+narrateur|Sa paume sent un peu le foin.
+papa|Tu as du foin, Mila ?
+enfant-f|Un peu, papa.
+narrateur|Maman tend le panier, vide et léger.
+enfant-f|Il est léger, maman.
+maman|Parce qu'il est vide.
+papa|Tu as vu le chat, Mila ?
+enfant-f|Il dort sous la table.
+papa|On le laisse.
+narrateur|Des voix passent, plus loin, sur la place.
+narrateur|Une petite balance fait tic, près de la caisse.
+enfant-f|Elle fait tic, maman.
+maman|C'est la balance, près des ronds.
+narrateur|Le bois de la table sent le soleil.
+enfant-f|Il est chaud, maman.
+maman|Et le plateau, lui, est froid.
+narrateur|Un filet de soleil tombe sur le bord.
+narrateur|Sur le bord, un éclat de panier brille.
+enfant-f|Il brille, papa !
+papa|Tu le vois, sur le panier ?
+enfant-f|Oui, près du bord.
+narrateur|Les ronds de la caisse sont pâles, un peu froids.
+enfant-f|Celui-là, papa.
+papa|Celui près de la queue ?
+enfant-f|Oui, le pâle.
+enfant-f|Je le veux, maintenant.
+narrateur|En ce moment, Mila avance vers la table.
+narrateur|La dame essuie le plateau de la balance.
+narrateur|Le métal est froid, malgré le soleil.
+enfant-f|Celui-là !
+narrateur|Mila parle trop vite vers la table.
+narrateur|Sa voix se mélange au tic de la balance.
+narrateur|La dame n'a pas levé les yeux.
+enfant-f|Oh.
+narrateur|Le rond pâle reste dans la caisse.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Je le prends !
+maman|Le fromage est sur la table.
+papa|Tu le vois, Mila ?
+narrateur|Les épaules de Mila tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>poule,paille</t>
+          <t>chat,balance</t>
         </is>
       </c>
     </row>
@@ -1395,27 +1417,27 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Mila veut l'œuf. Que dit-elle ?</t>
+          <t>Mila parle à la dame. Quels mots dit-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Mila veut l'œuf. Que dit-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila parle à la &lt;emphasis level="moderate"&gt;dame&lt;/emphasis&gt;. Quels mots dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Honoré parle à la dame. Quels mots dit-il ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila parle à la &lt;emphasis&gt;dame&lt;/emphasis&gt;. Quels mots dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>s'il te plaît</t>
+          <t>bonjour</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>s'il te plaît | merci | bonjour | s'il te plait</t>
+          <t>bonjour | s'il te plaît | merci | bonjour merci</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1430,7 +1452,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Elle dit s'il te plaît. Que dit Mila ?</t>
+          <t>Elle dit bonjour. Quels mots dit Mila ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1468,18 +1490,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1494,34 +1516,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>dame</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1530,29 +1556,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_dit_bonjour_a_la_dame; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Mila veut l'œuf.
-narrateur|Que dit-elle ?</t>
+          <t>narrateur|Mila parle à la dame.
+narrateur|Quels mots dit-elle ?</t>
         </is>
       </c>
     </row>
@@ -1579,17 +1605,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. L'œuf brun, s'il te plaît. Celui du nid. La dame glisse la main sous la paille. Elle pose l'œuf sur le torchon. Le torchon se creuse un peu. Merci. Merci. Il est chaud, maman. Comme un petit soleil. Mila pose les deux mains autour. La chaleur passe à travers le linge. Plus loin, une chèvre sonne sa cloche. Le lait attend dans un pot de verre. Un peu de lait, pour la pâte ? Oui. Ils s'arrêtent près de la barrière. Bonjour. Un peu de lait, s'il te plaît. La dame verse le lait, tout blanc. Le pot devient lourd dans le panier. Merci. Tu as demandé deux fois. Bravo, Mila. La poule picore encore, derrière eux. La cloche de la chèvre s'éloigne.</t>
+          <t>Mila avance trop vite vers la table. Celui-là, maintenant ! Sa voix se mélange au tic. Oh. Le rond pâle reste dans la caisse. La dame essuie, sans lever les yeux. Mila refuse de foncer. Elle referme la main sur le panier. Elle écoute la balance, un instant. Tu veux venir près de la table ? Papa s'accroupit à la même hauteur. Mila pose un pied près du bois. Le plateau de la balance est froid. Bonjour. Celui-là. S'il te plaît. La dame pose le chiffon. Elle lève les yeux. Une main coupe un rond pâle. La petite balance fait tic. Elle glisse le rond dans le panier. Le papier est froid, un peu gras. Merci, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Les épaules se relèvent un peu. Tu as les mains au frais ? Un peu, maman. Ça sent le lait, près d'elle. Le fromage est à moi. Il est dans ton panier. Mila pose une main sur le bord. Le bord est un peu rêche. Sur le bord, un éclat de panier tient. La balance se tait.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. L'œuf brun, s'il te plaît. Celui du nid. La dame glisse la main sous la paille. Elle pose l'œuf sur le torchon. Le torchon se creuse un peu. Merci. Merci. Il est chaud, maman. Comme un petit soleil. Mila pose les deux mains autour. La chaleur passe à travers le linge. Plus loin, une chèvre sonne sa cloche. Le lait attend dans un pot de verre. Un peu de lait, pour la pâte ? Oui. Ils s'arrêtent près de la barrière. Bonjour. Un peu de lait, s'il te plaît. La dame verse le lait, tout blanc. Le pot devient lourd dans le panier. Merci. Tu as demandé deux fois. Bravo, Mila. La poule picore encore, derrière eux. La cloche de la chèvre s'éloigne.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila avance trop vite vers la table. Celui-là, maintenant ! Sa voix se mélange au tic. Oh. Le rond pâle reste dans la caisse. La dame essuie, sans lever les yeux. Mila refuse de foncer. Elle referme la main sur le panier. Elle écoute la balance, un instant. Tu veux venir près de la table ? Papa s'accroupit à la même hauteur. Mila pose un pied près du bois. Le plateau de la balance est froid. &lt;emphasis level="moderate"&gt;Bonjour&lt;/emphasis&gt;. Celui-là. S'il te plaît. La dame pose le chiffon. Elle lève les yeux. Une main coupe un rond pâle. La petite balance fait tic. Elle glisse le rond dans le panier. Le papier est froid, un peu gras. Merci, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Les épaules se relèvent un peu. Tu as les mains au frais ? Un peu, maman. Ça sent le lait, près d'elle. Le fromage est à moi. Il est dans ton panier. Mila pose une main sur le bord. Le bord est un peu rêche. Sur le bord, un éclat de panier tient. La balance se tait.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Honoré a dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Il a dit s'il te plaît. Il a dit merci. Maman était là. [pause]</t>
+          <t>Mila avance trop vite vers la table. Celui-là, maintenant ! Sa voix se mélange au tic. Oh. Le rond pâle reste dans la caisse. La dame essuie, sans lever les yeux. Mila refuse de foncer. Elle referme la main sur le panier. Elle écoute la balance, un instant. Tu veux venir près de la table ? Papa s'accroupit à la même hauteur. Mila pose un pied près du bois. Le plateau de la balance est froid. &lt;emphasis&gt;Bonjour&lt;/emphasis&gt;. Celui-là. S'il te plaît. La dame pose le chiffon. Elle lève les yeux. Une main coupe un rond pâle. La petite balance fait tic. Elle glisse le rond dans le panier. Le papier est froid, un peu gras. Merci, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Les épaules se relèvent un peu. Tu as les mains au frais ? Un peu, maman. Ça sent le lait, près d'elle. Le fromage est à moi. Il est dans ton panier. Mila pose une main sur le bord. Le bord est un peu rêche. Sur le bord, un éclat de panier tient. La balance se tait. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1636,7 +1662,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1644,10 +1670,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1670,30 +1696,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>Bonjour</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1702,10 +1728,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1718,43 +1744,51 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=bonjour_ouvre_le_panier; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-f|Bonjour.
-maman|Bonjour.
-enfant-f|L'œuf brun, s'il te plaît.
-enfant-f|Celui du nid.
-narrateur|La dame glisse la main sous la paille.
-narrateur|Elle pose l'œuf sur le torchon.
-narrateur|Le torchon se creuse un peu.
-enfant-f|Merci.
-maman|Merci.
-enfant-f|Il est chaud, maman.
-maman|Comme un petit soleil.
-narrateur|Mila pose les deux mains autour.
-narrateur|La chaleur passe à travers le linge.
-narrateur|Plus loin, une chèvre sonne sa cloche.
-narrateur|Le lait attend dans un pot de verre.
-maman|Un peu de lait, pour la pâte ?
-enfant-f|Oui.
-narrateur|Ils s'arrêtent près de la barrière.
+          <t>narrateur|Mila avance trop vite vers la table.
+enfant-f|Celui-là, maintenant !
+narrateur|Sa voix se mélange au tic.
+enfant-f|Oh.
+narrateur|Le rond pâle reste dans la caisse.
+narrateur|La dame essuie, sans lever les yeux.
+narrateur|Mila refuse de foncer.
+narrateur|Elle referme la main sur le panier.
+narrateur|Elle écoute la balance, un instant.
+papa|Tu veux venir près de la table ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Mila pose un pied près du bois.
+narrateur|Le plateau de la balance est froid.
 enfant-f|Bonjour.
-enfant-f|Un peu de lait, s'il te plaît.
-narrateur|La dame verse le lait, tout blanc.
-narrateur|Le pot devient lourd dans le panier.
-enfant-f|Merci.
-maman|Tu as demandé deux fois.
-maman|Bravo, Mila.
-narrateur|La poule picore encore, derrière eux.
-narrateur|La cloche de la chèvre s'éloigne.</t>
+enfant-f|Celui-là.
+enfant-f|S'il te plaît.
+narrateur|La dame pose le chiffon.
+narrateur|Elle lève les yeux.
+narrateur|Une main coupe un rond pâle.
+narrateur|La petite balance fait tic.
+narrateur|Elle glisse le rond dans le panier.
+narrateur|Le papier est froid, un peu gras.
+papa|Merci, Mila.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Mila se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tu as les mains au frais ?
+enfant-f|Un peu, maman.
+narrateur|Ça sent le lait, près d'elle.
+enfant-f|Le fromage est à moi.
+maman|Il est dans ton panier.
+narrateur|Mila pose une main sur le bord.
+narrateur|Le bord est un peu rêche.
+narrateur|Sur le bord, un éclat de panier tient.
+narrateur|La balance se tait.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>cloche</t>
+          <t>papier,balance</t>
         </is>
       </c>
     </row>
@@ -1781,17 +1815,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sur le chemin, le panier penche un peu. L'œuf roule contre le pot, tout doux. Il est encore chaud. On marche sans sauter. La paille laisse une odeur sur les sandales. À la maison, papa a déjà le saladier. Vous avez l'œuf ? Oui, papa. Il était dans le nid. Il sent la paille, encore. Et le lait est là. Papa casse l'œuf au-dessus du bol. Le jaune tombe, tout rond. C'est pour le gâteau. Tu l'as demandé, Mila ? Bonjour. S'il te plaît. Merci. Le gâteau va sentir la ferme. Un peu le grain, un peu le lait. La plume du loquet n'est plus là. Le saladier est jaune, maintenant.</t>
+          <t>Mila lève le panier trop vite. Je le montre, d'un coup ! Le bord penche entre les doigts. Le fromage penche vers le chat. Oh. Mila avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Mila refuse de foncer, cette fois. Elle observe le panier, écoute le marché. Sur le bord, un éclat de panier luit. Là, près du bord. Mila tient le panier des deux mains. Le bord est rêche, un peu froid. Il est froid, papa. Tu le portes jusqu'à la place ? Oui, papa. On marche ? Oui, maman. Le chat ouvre un œil, puis se recouche. Il dort. On le laisse. Mila serre le panier contre elle. Le fromage reste. Le panier penche, puis se cale. Je le tiens. On avance. Mila passe près de la table. La caisse reste derrière.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sur le chemin, le panier penche un peu. L'œuf roule contre le pot, tout doux. Il est encore chaud. On marche sans sauter. La paille laisse une odeur sur les sandales. À la maison, papa a déjà le saladier. Vous avez l'œuf ? Oui, papa. Il était dans le nid. Il sent la paille, encore. Et le lait est là. Papa casse l'œuf au-dessus du bol. Le jaune tombe, tout rond. C'est pour le gâteau. Tu l'as demandé, Mila ? Bonjour. S'il te plaît. Merci. Le gâteau va sentir la ferme. Un peu le grain, un peu le lait. La plume du loquet n'est plus là. Le saladier est jaune, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila lève le panier trop vite. Je le montre, d'un coup ! Le bord penche entre les doigts. Le fromage penche vers le chat. Oh. Mila avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Mila refuse de foncer, cette fois. Elle observe le panier, écoute le marché. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de panier&lt;/emphasis&gt; luit. Là, près du bord. Mila tient le panier des deux mains. Le bord est rêche, un peu froid. Il est froid, papa. Tu le portes jusqu'à la place ? Oui, papa. On marche ? Oui, maman. Le chat ouvre un œil, puis se recouche. Il dort. On le laisse. Mila serre le panier contre elle. Le fromage reste. Le panier penche, puis se cale. Je le tiens. On avance. Mila passe près de la table. La caisse reste derrière.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Honoré croque la pomme. Maman dit &lt;emphasis&gt;merci&lt;/emphasis&gt; aussi. [pause]</t>
+          <t>&lt;low-pitch&gt;Mila lève le panier trop vite. Je le montre, d'un coup ! Le bord penche entre les doigts. Le fromage penche vers le chat. Oh. Mila avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Mila refuse de foncer, cette fois. Elle observe le panier, écoute le marché. Sur le bord, un &lt;emphasis&gt;éclat de panier&lt;/emphasis&gt; luit. Là, près du bord. Mila tient le panier des deux mains. Le bord est rêche, un peu froid. Il est froid, papa. Tu le portes jusqu'à la place ? Oui, papa. On marche ? Oui, maman. Le chat ouvre un œil, puis se recouche. Il dort. On le laisse. Mila serre le panier contre elle. Le fromage reste. Le panier penche, puis se cale. Je le tiens. On avance. Mila passe près de la table. La caisse reste derrière.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1838,7 +1872,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1846,22 +1880,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1872,30 +1910,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>merci</t>
+          <t>éclat de panier</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1904,50 +1942,62 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat_de_panier; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sur le chemin, le panier penche un peu.
-narrateur|L'œuf roule contre le pot, tout doux.
-enfant-f|Il est encore chaud.
-maman|On marche sans sauter.
-narrateur|La paille laisse une odeur sur les sandales.
-narrateur|À la maison, papa a déjà le saladier.
-papa|Vous avez l'œuf ?
+          <t>narrateur|Mila lève le panier trop vite.
+enfant-f|Je le montre, d'un coup !
+narrateur|Le bord penche entre les doigts.
+narrateur|Le fromage penche vers le chat.
+enfant-f|Oh.
+narrateur|Mila avance les mains.
+narrateur|Puis elle s'arrête net.
+enfant-f|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Mila refuse de foncer, cette fois.
+narrateur|Elle observe le panier, écoute le marché.
+narrateur|Sur le bord, un éclat de panier luit.
+enfant-f|Là, près du bord.
+narrateur|Mila tient le panier des deux mains.
+narrateur|Le bord est rêche, un peu froid.
+enfant-f|Il est froid, papa.
+papa|Tu le portes jusqu'à la place ?
 enfant-f|Oui, papa.
-enfant-f|Il était dans le nid.
-papa|Il sent la paille, encore.
-maman|Et le lait est là.
-narrateur|Papa casse l'œuf au-dessus du bol.
-narrateur|Le jaune tombe, tout rond.
-enfant-f|C'est pour le gâteau.
-papa|Tu l'as demandé, Mila ?
-enfant-f|Bonjour.
-enfant-f|S'il te plaît.
-enfant-f|Merci.
-papa|Le gâteau va sentir la ferme.
-maman|Un peu le grain, un peu le lait.
-narrateur|La plume du loquet n'est plus là.
-narrateur|Le saladier est jaune, maintenant.</t>
+maman|On marche ?
+enfant-f|Oui, maman.
+narrateur|Le chat ouvre un œil, puis se recouche.
+enfant-f|Il dort.
+papa|On le laisse.
+narrateur|Mila serre le panier contre elle.
+enfant-f|Le fromage reste.
+narrateur|Le panier penche, puis se cale.
+enfant-f|Je le tiens.
+maman|On avance.
+narrateur|Mila passe près de la table.
+narrateur|La caisse reste derrière.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>bol,pas</t>
+          <t>panier,pas</t>
         </is>
       </c>
     </row>
@@ -1974,17 +2024,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le saladier repose sur la table. L'œuf n'est plus dans le nid. Bonne après-midi, Mila. Le gâteau va cuire.</t>
+          <t>Le panier brillait, papa. Tu le vois, comme à la table ? Oui, sur le bord. Mila pose le panier contre son bras. On le garde au frais ? Oui, maman. Le lait sentait bon. Il est contre toi. Une odeur de foin reste dans le panier. Mila respire, plus large. On rentre ? Oui. Les joues de Mila se réchauffent. Le panier reste froid sous la main. Le chat dort sous la table. Il n'a pas bougé. Comme tout à l'heure ? Oui, maman. Le soleil est sur le bord, toi ? Oui, papa. Un éclat de panier reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le saladier repose sur la table. L'œuf n'est plus dans le nid. Bonne après-midi, Mila. Le gâteau va cuire.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le panier brillait, papa. Tu le vois, comme à la table ? Oui, sur le bord. Mila pose le panier contre son bras. On le garde au frais ? Oui, maman. Le lait sentait bon. Il est contre toi. Une odeur de foin reste dans le panier. Mila respire, plus large. On rentre ? Oui. Les joues de Mila se réchauffent. Le panier reste froid sous la main. Le chat dort sous la table. Il n'a pas bougé. Comme tout à l'heure ? Oui, maman. Le soleil est sur le bord, toi ? Oui, papa. Un &lt;emphasis level="moderate"&gt;éclat de panier&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le panier brillait, papa. Tu le vois, comme à la table ? Oui, sur le bord. Mila pose le panier contre son bras. On le garde au frais ? Oui, maman. Le lait sentait bon. Il est contre toi. Une odeur de foin reste dans le panier. Mila respire, plus large. On rentre ? Oui. Les joues de Mila se réchauffent. Le panier reste froid sous la main. Le chat dort sous la table. Il n'a pas bougé. Comme tout à l'heure ? Oui, maman. Le soleil est sur le bord, toi ? Oui, papa. Un &lt;emphasis&gt;éclat de panier&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2031,18 +2081,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2051,12 +2101,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2065,17 +2115,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de panier</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2084,11 +2138,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2097,27 +2151,53 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_panier_reste_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le saladier repose sur la table.
-narrateur|L'œuf n'est plus dans le nid.
-maman|Bonne après-midi, Mila.
-papa|Le gâteau va cuire.</t>
+          <t>enfant-f|Le panier brillait, papa.
+papa|Tu le vois, comme à la table ?
+enfant-f|Oui, sur le bord.
+narrateur|Mila pose le panier contre son bras.
+maman|On le garde au frais ?
+enfant-f|Oui, maman.
+enfant-f|Le lait sentait bon.
+maman|Il est contre toi.
+narrateur|Une odeur de foin reste dans le panier.
+narrateur|Mila respire, plus large.
+papa|On rentre ?
+enfant-f|Oui.
+narrateur|Les joues de Mila se réchauffent.
+narrateur|Le panier reste froid sous la main.
+narrateur|Le chat dort sous la table.
+enfant-f|Il n'a pas bougé.
+maman|Comme tout à l'heure ?
+enfant-f|Oui, maman.
+papa|Le soleil est sur le bord, toi ?
+enfant-f|Oui, papa.
+narrateur|Un éclat de panier reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pas</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2195,6 +2275,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>